<commit_message>
Add Br5161 as fourth pick for E4+ EA Xenium dononr
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/04_xenium_donors/xenium_donor_picks_tissue_inventory.xlsx
+++ b/processed-data/21_Xenium/04_xenium_donors/xenium_donor_picks_tissue_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/21_Xenium/04_xenium_donors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="8_{9C96362F-A148-F34A-B3A2-4E10A0490E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{258177CD-3A22-8342-96C6-F89790FCEFCC}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{9C96362F-A148-F34A-B3A2-4E10A0490E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{270CDB38-3324-C545-B7A7-061D8C0CB6FD}"/>
   <bookViews>
     <workbookView xWindow="1060" yWindow="660" windowWidth="27640" windowHeight="16680" xr2:uid="{516D38BB-D242-7945-94E2-0EDD02C8CBFA}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="50">
   <si>
     <t>BrNum</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t>small Visium sample</t>
+  </si>
+  <si>
+    <t>Br5161 E4+          E4/E4 EA       M      54.4 FALSE FALSE       FALSE          0     4</t>
   </si>
 </sst>
 </file>
@@ -743,16 +746,6 @@
   <dxfs count="3">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -771,6 +764,16 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -782,6 +785,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1101,9 +1108,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C4EF1EA-A7AD-C74F-86EA-F1C14CDD47D7}">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
     <col min="12" max="12" width="15.1640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="18.5" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="17.1640625" bestFit="1" customWidth="1"/>
@@ -1872,15 +1880,20 @@
         <v>1</v>
       </c>
     </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O17" xr:uid="{6C4EF1EA-A7AD-C74F-86EA-F1C14CDD47D7}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O17">
       <sortCondition ref="B1:B17"/>
     </sortState>
   </autoFilter>
-  <conditionalFormatting sqref="O2:O17">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
-      <formula>TRUE</formula>
+  <conditionalFormatting sqref="E2:E17">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:I17">
@@ -1888,9 +1901,9 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E17">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
-      <formula>"F"</formula>
+  <conditionalFormatting sqref="O2:O17">
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="equal">
+      <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix deletion of modeling_results
</commit_message>
<xml_diff>
--- a/processed-data/21_Xenium/04_xenium_donors/xenium_donor_picks_tissue_inventory.xlsx
+++ b/processed-data/21_Xenium/04_xenium_donors/xenium_donor_picks_tissue_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lieberinstitute-my.sharepoint.com/personal/louise_huuki_libd_org/Documents/LIBD_code/LFF_spatial_ERC/processed-data/21_Xenium/04_xenium_donors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="8_{9C96362F-A148-F34A-B3A2-4E10A0490E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{270CDB38-3324-C545-B7A7-061D8C0CB6FD}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{9C96362F-A148-F34A-B3A2-4E10A0490E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D57A145C-1693-7B45-9F0B-E70359EA4FC8}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="660" windowWidth="27640" windowHeight="16680" xr2:uid="{516D38BB-D242-7945-94E2-0EDD02C8CBFA}"/>
+    <workbookView xWindow="32420" yWindow="1720" windowWidth="27640" windowHeight="16680" xr2:uid="{516D38BB-D242-7945-94E2-0EDD02C8CBFA}"/>
   </bookViews>
   <sheets>
     <sheet name="xenium_donor_picks" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="50">
   <si>
     <t>BrNum</t>
   </si>
@@ -172,7 +172,7 @@
     <t>small Visium sample</t>
   </si>
   <si>
-    <t>Br5161 E4+          E4/E4 EA       M      54.4 FALSE FALSE       FALSE          0     4</t>
+    <t>Br5161</t>
   </si>
 </sst>
 </file>
@@ -1884,6 +1884,42 @@
       <c r="A18" t="s">
         <v>49</v>
       </c>
+      <c r="B18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18">
+        <v>54.4</v>
+      </c>
+      <c r="G18" t="b">
+        <v>0</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>4</v>
+      </c>
+      <c r="L18" t="s">
+        <v>38</v>
+      </c>
+      <c r="M18" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O17" xr:uid="{6C4EF1EA-A7AD-C74F-86EA-F1C14CDD47D7}">

</xml_diff>